<commit_message>
stage3g: promote approved draft overrides to official 02b
</commit_message>
<xml_diff>
--- a/data/overrides/02B_ai_repair_override.xlsx
+++ b/data/overrides/02B_ai_repair_override.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ai_repair_override" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ai_repair_override" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,96 +425,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>repair_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>asset_package</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>standard_metric</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>year</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>final_value</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>final_unit</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>final_value_source</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>final_review_status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>evidence</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>source_reference</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>approval_review_file</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>real_apply_log_file</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>real_apply_diff_file</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>stage_name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>apply_batch_id</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>created_from_commit</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>provenance_status</t>
         </is>
@@ -534,10 +546,8 @@
           <t>2025A</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1640.2</t>
-        </is>
+      <c r="F2" t="n">
+        <v>1640.2</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -626,10 +636,8 @@
           <t>2026E</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>1860.07</t>
-        </is>
+      <c r="F3" t="n">
+        <v>1860.07</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -718,10 +726,8 @@
           <t>2027E</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>2064.58</t>
-        </is>
+      <c r="F4" t="n">
+        <v>2064.58</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -810,10 +816,8 @@
           <t>2028E</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2292.66</t>
-        </is>
+      <c r="F5" t="n">
+        <v>2292.66</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -902,10 +906,8 @@
           <t>2025A</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>3.71</t>
-        </is>
+      <c r="F6" t="n">
+        <v>3.71</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -990,10 +992,8 @@
           <t>2026E</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>3.18</t>
-        </is>
+      <c r="F7" t="n">
+        <v>3.18</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
@@ -1078,10 +1078,8 @@
           <t>2027E</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2.75</t>
-        </is>
+      <c r="F8" t="n">
+        <v>2.75</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
@@ -1166,10 +1164,8 @@
           <t>2028E</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2.38</t>
-        </is>
+      <c r="F9" t="n">
+        <v>2.38</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
@@ -1254,10 +1250,8 @@
           <t>2025A</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>11.16</t>
-        </is>
+      <c r="F10" t="n">
+        <v>11.16</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -1342,10 +1336,8 @@
           <t>2026E</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10.72</t>
-        </is>
+      <c r="F11" t="n">
+        <v>10.72</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
@@ -1430,10 +1422,8 @@
           <t>2027E</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>9.15</t>
-        </is>
+      <c r="F12" t="n">
+        <v>9.15</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
@@ -1518,10 +1508,8 @@
           <t>2028E</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>7.72</t>
-        </is>
+      <c r="F13" t="n">
+        <v>7.72</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
@@ -1606,10 +1594,8 @@
           <t>2025</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>21.3</t>
-        </is>
+      <c r="F14" t="n">
+        <v>21.3</v>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
@@ -1665,6 +1651,326 @@
       <c r="R14" t="inlineStr">
         <is>
           <t>REBUILDABLE_INPUT_READY</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>STAGE3G_PROMOTED_REVIEW_BEFORE_APPLY_1896910f</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>REVIEW_BEFORE_APPLY_1896910f</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>H3_AP202605141822317484_1_资产包</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>每股收益</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025A</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.51</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>元/股</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>stage3_ai_repair_override</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>approved_promoted</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>D:\_datefac\output\stage3f_draft_promotion_approval\95_stage3f_draft_promotion_approval.xlsx</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>stage3_draft_override_promotion</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>stage3g_promote_20260520_222137</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>PROMOTED_TO_OFFICIAL_02B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>STAGE3G_PROMOTED_REVIEW_BEFORE_APPLY_d6c94fa3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>REVIEW_BEFORE_APPLY_d6c94fa3</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>H3_AP202605141822317484_1_资产包</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>每股收益</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>元/股</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>stage3_ai_repair_override</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>approved_promoted</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>D:\_datefac\output\stage3f_draft_promotion_approval\95_stage3f_draft_promotion_approval.xlsx</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>stage3_draft_override_promotion</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>stage3g_promote_20260520_222137</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>PROMOTED_TO_OFFICIAL_02B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>STAGE3G_PROMOTED_REVIEW_BEFORE_APPLY_b5b308bc</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>REVIEW_BEFORE_APPLY_b5b308bc</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>H3_AP202605141822317484_1_资产包</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>每股收益</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2027E</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>元/股</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>stage3_ai_repair_override</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>approved_promoted</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>D:\_datefac\output\stage3f_draft_promotion_approval\95_stage3f_draft_promotion_approval.xlsx</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>stage3_draft_override_promotion</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>stage3g_promote_20260520_222137</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>PROMOTED_TO_OFFICIAL_02B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>STAGE3G_PROMOTED_REVIEW_BEFORE_APPLY_1ef7d21b</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>REVIEW_BEFORE_APPLY_1ef7d21b</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>H3_AP202605141822317484_1_资产包</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>每股收益</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2028E</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.71</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>元/股</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>stage3_ai_repair_override</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>approved_promoted</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>S1|p005|t001|r047</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>D:\_datefac\output\stage3f_draft_promotion_approval\95_stage3f_draft_promotion_approval.xlsx</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>stage3_draft_override_promotion</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>stage3g_promote_20260520_222137</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>PROMOTED_TO_OFFICIAL_02B</t>
         </is>
       </c>
     </row>

</xml_diff>